<commit_message>
feat: implement attribute-based data validation system with support for custom rules and context-aware checks
</commit_message>
<xml_diff>
--- a/Documents/Excel/CityTest.xlsx
+++ b/Documents/Excel/CityTest.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\SeanProjects\CustomPackages\ExcelExtruder\Documents\Excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CF9E4760-B34D-44FB-AA25-5EA87A9E69FF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DC368855-EC3E-419B-BBBA-E3AE14F79A51}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="783" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="783" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="sCityVO" sheetId="6" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="127" uniqueCount="108">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="133" uniqueCount="108">
   <si>
     <t>#</t>
   </si>
@@ -96,9 +96,6 @@
     <t>苏州府印</t>
   </si>
   <si>
-    <t>Map2</t>
-  </si>
-  <si>
     <t>C3</t>
   </si>
   <si>
@@ -157,9 +154,6 @@
   </si>
   <si>
     <t>Map7</t>
-  </si>
-  <si>
-    <t>C8</t>
   </si>
   <si>
     <t>绍兴府</t>
@@ -368,6 +362,14 @@
   </si>
   <si>
     <t>m_exp</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>C8</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Map12</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
 </sst>
@@ -736,7 +738,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6B4CF102-FCD0-4C03-97A2-6BA18FF3CB38}">
-  <dimension ref="A1:G19"/>
+  <dimension ref="A1:G20"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="3.25" style="3" customWidth="1"/>
@@ -764,33 +766,33 @@
         <v>10</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A2" s="3" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="B2" s="4" t="s">
         <v>11</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="E2" s="4" t="s">
         <v>12</v>
       </c>
       <c r="F2" s="4" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="G2" s="4" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.2">
@@ -807,10 +809,10 @@
         <v>16</v>
       </c>
       <c r="F3" s="4" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="G3" s="4" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.2">
@@ -824,254 +826,254 @@
         <v>19</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>20</v>
+        <v>107</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="G4" s="4" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.2">
       <c r="B5" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="C5" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="C5" s="4" t="s">
+      <c r="D5" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="D5" s="4" t="s">
+      <c r="E5" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="E5" s="4" t="s">
-        <v>24</v>
-      </c>
       <c r="F5" s="4" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="G5" s="4" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.2">
       <c r="B6" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="C6" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="C6" s="4" t="s">
+      <c r="D6" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="D6" s="4" t="s">
+      <c r="E6" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="E6" s="4" t="s">
-        <v>28</v>
-      </c>
       <c r="F6" s="4" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="G6" s="4" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.2">
       <c r="B7" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="C7" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="C7" s="4" t="s">
+      <c r="D7" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="D7" s="4" t="s">
+      <c r="E7" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="E7" s="4" t="s">
-        <v>32</v>
-      </c>
       <c r="F7" s="4" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="G7" s="4" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.2">
       <c r="B8" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="C8" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="C8" s="4" t="s">
+      <c r="D8" s="4" t="s">
         <v>34</v>
       </c>
-      <c r="D8" s="4" t="s">
+      <c r="E8" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="E8" s="4" t="s">
-        <v>36</v>
-      </c>
       <c r="F8" s="4" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="G8" s="4" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.2">
       <c r="B9" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="C9" s="4" t="s">
         <v>37</v>
       </c>
-      <c r="C9" s="4" t="s">
+      <c r="D9" s="4" t="s">
         <v>38</v>
       </c>
-      <c r="D9" s="4" t="s">
+      <c r="E9" s="4" t="s">
         <v>39</v>
       </c>
-      <c r="E9" s="4" t="s">
-        <v>40</v>
-      </c>
       <c r="F9" s="4" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="G9" s="4" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.2">
       <c r="B10" s="4" t="s">
+        <v>106</v>
+      </c>
+      <c r="C10" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="D10" s="4" t="s">
         <v>41</v>
       </c>
-      <c r="C10" s="4" t="s">
+      <c r="E10" s="4" t="s">
         <v>42</v>
       </c>
-      <c r="D10" s="4" t="s">
-        <v>43</v>
-      </c>
-      <c r="E10" s="4" t="s">
-        <v>44</v>
-      </c>
       <c r="F10" s="4" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="G10" s="4" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.2">
       <c r="B11" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="C11" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="D11" s="4" t="s">
         <v>45</v>
       </c>
-      <c r="C11" s="4" t="s">
+      <c r="E11" s="4" t="s">
         <v>46</v>
       </c>
-      <c r="D11" s="4" t="s">
-        <v>47</v>
-      </c>
-      <c r="E11" s="4" t="s">
-        <v>48</v>
-      </c>
       <c r="F11" s="4" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="G11" s="4" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.2">
       <c r="B12" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="C12" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="D12" s="4" t="s">
         <v>49</v>
       </c>
-      <c r="C12" s="4" t="s">
+      <c r="E12" s="4" t="s">
         <v>50</v>
       </c>
-      <c r="D12" s="4" t="s">
-        <v>51</v>
-      </c>
-      <c r="E12" s="4" t="s">
-        <v>52</v>
-      </c>
       <c r="F12" s="4" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="G12" s="4" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.2">
       <c r="B13" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="C13" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="D13" s="4" t="s">
         <v>53</v>
       </c>
-      <c r="C13" s="4" t="s">
+      <c r="E13" s="4" t="s">
         <v>54</v>
       </c>
-      <c r="D13" s="4" t="s">
-        <v>55</v>
-      </c>
-      <c r="E13" s="4" t="s">
-        <v>56</v>
-      </c>
       <c r="F13" s="4" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="G13" s="4" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.2">
       <c r="B14" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="C14" s="4" t="s">
+        <v>56</v>
+      </c>
+      <c r="D14" s="4" t="s">
         <v>57</v>
       </c>
-      <c r="C14" s="4" t="s">
+      <c r="E14" s="4" t="s">
         <v>58</v>
       </c>
-      <c r="D14" s="4" t="s">
-        <v>59</v>
-      </c>
-      <c r="E14" s="4" t="s">
-        <v>60</v>
-      </c>
       <c r="F14" s="4" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="G14" s="4" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
     </row>
     <row r="15" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B15" s="4" t="s">
+        <v>59</v>
+      </c>
+      <c r="C15" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="D15" s="4" t="s">
         <v>61</v>
       </c>
-      <c r="C15" s="4" t="s">
+      <c r="E15" s="4" t="s">
         <v>62</v>
       </c>
-      <c r="D15" s="4" t="s">
-        <v>63</v>
-      </c>
-      <c r="E15" s="4" t="s">
-        <v>64</v>
-      </c>
       <c r="F15" s="4" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="G15" s="4" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A16" s="1"/>
       <c r="B16" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="C16" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="D16" s="4" t="s">
         <v>65</v>
       </c>
-      <c r="C16" s="4" t="s">
+      <c r="E16" s="4" t="s">
         <v>66</v>
       </c>
-      <c r="D16" s="4" t="s">
-        <v>67</v>
-      </c>
-      <c r="E16" s="4" t="s">
-        <v>68</v>
-      </c>
       <c r="F16" s="4" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="G16" s="4" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.2">
@@ -1079,22 +1081,22 @@
         <v>0</v>
       </c>
       <c r="B17" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="C17" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="D17" s="4" t="s">
         <v>69</v>
       </c>
-      <c r="C17" s="4" t="s">
+      <c r="E17" s="4" t="s">
         <v>70</v>
       </c>
-      <c r="D17" s="4" t="s">
-        <v>71</v>
-      </c>
-      <c r="E17" s="4" t="s">
-        <v>72</v>
-      </c>
       <c r="F17" s="4" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="G17" s="4" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.2">
@@ -1102,42 +1104,62 @@
         <v>0</v>
       </c>
       <c r="B18" s="4" t="s">
+        <v>71</v>
+      </c>
+      <c r="C18" s="4" t="s">
+        <v>72</v>
+      </c>
+      <c r="D18" s="4" t="s">
         <v>73</v>
       </c>
-      <c r="C18" s="4" t="s">
+      <c r="E18" s="4" t="s">
         <v>74</v>
       </c>
-      <c r="D18" s="4" t="s">
-        <v>75</v>
-      </c>
-      <c r="E18" s="4" t="s">
-        <v>76</v>
-      </c>
       <c r="F18" s="4" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="G18" s="4" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.2">
       <c r="B19" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="C19" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="D19" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="E19" s="4" t="s">
         <v>77</v>
       </c>
-      <c r="C19" s="4" t="s">
-        <v>78</v>
-      </c>
-      <c r="D19" s="4" t="s">
-        <v>78</v>
-      </c>
-      <c r="E19" s="4" t="s">
-        <v>79</v>
-      </c>
       <c r="F19" s="4" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="G19" s="4" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="B20" s="4" t="s">
         <v>106</v>
+      </c>
+      <c r="C20" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="D20" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="E20" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="F20" s="4" t="s">
+        <v>81</v>
+      </c>
+      <c r="G20" s="4" t="s">
+        <v>90</v>
       </c>
     </row>
   </sheetData>
@@ -1182,13 +1204,13 @@
     </row>
     <row r="2" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A2" s="5" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="B2" s="6" t="s">
         <v>2</v>
       </c>
       <c r="C2" s="6" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="D2" s="6"/>
       <c r="E2" s="6"/>
@@ -1202,7 +1224,8 @@
         <v>0</v>
       </c>
       <c r="C3" s="4">
-        <v>-100</v>
+        <f t="shared" ref="C3:C5" si="0">ROUND(E3*(3+D3),0)</f>
+        <v>0</v>
       </c>
       <c r="D3" s="4">
         <v>0</v>
@@ -1214,7 +1237,7 @@
         <v>3</v>
       </c>
       <c r="G3" s="4">
-        <f t="shared" ref="G3:G32" si="0">F3*3</f>
+        <f t="shared" ref="G3:G32" si="1">F3*3</f>
         <v>9</v>
       </c>
       <c r="H3" s="4"/>
@@ -1223,6 +1246,10 @@
       <c r="B4" s="4">
         <v>1</v>
       </c>
+      <c r="C4" s="4">
+        <f t="shared" si="0"/>
+        <v>20</v>
+      </c>
       <c r="D4" s="4">
         <v>1</v>
       </c>
@@ -1233,7 +1260,7 @@
         <v>4</v>
       </c>
       <c r="G4" s="4">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>12</v>
       </c>
       <c r="H4" s="4"/>
@@ -1243,6 +1270,7 @@
         <v>2</v>
       </c>
       <c r="C5" s="4">
+        <f t="shared" si="0"/>
         <v>140</v>
       </c>
       <c r="D5" s="4">
@@ -1255,7 +1283,7 @@
         <v>5</v>
       </c>
       <c r="G5" s="4">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>15</v>
       </c>
       <c r="H5" s="4"/>
@@ -1265,7 +1293,7 @@
         <v>3</v>
       </c>
       <c r="C6" s="4">
-        <f t="shared" ref="C5:C32" si="1">ROUND(E6*(3+D6),0)</f>
+        <f t="shared" ref="C6:C32" si="2">ROUND(E6*(3+D6),0)</f>
         <v>210</v>
       </c>
       <c r="D6" s="4">
@@ -1278,7 +1306,7 @@
         <v>6</v>
       </c>
       <c r="G6" s="4">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>18</v>
       </c>
       <c r="H6" s="4"/>
@@ -1288,7 +1316,7 @@
         <v>4</v>
       </c>
       <c r="C7" s="4">
-        <f t="shared" si="1"/>
+        <f>ROUND(E7*(3+D7),0)</f>
         <v>270</v>
       </c>
       <c r="D7" s="4">
@@ -1301,7 +1329,7 @@
         <v>7</v>
       </c>
       <c r="G7" s="4">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>21</v>
       </c>
       <c r="H7" s="4"/>
@@ -1311,7 +1339,7 @@
         <v>5</v>
       </c>
       <c r="C8" s="4">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>300</v>
       </c>
       <c r="D8" s="4">
@@ -1324,7 +1352,7 @@
         <v>8</v>
       </c>
       <c r="G8" s="4">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>24</v>
       </c>
       <c r="H8" s="4"/>
@@ -1334,7 +1362,7 @@
         <v>6</v>
       </c>
       <c r="C9" s="4">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>429</v>
       </c>
       <c r="D9" s="4">
@@ -1347,7 +1375,7 @@
         <v>9</v>
       </c>
       <c r="G9" s="4">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>27</v>
       </c>
     </row>
@@ -1356,7 +1384,7 @@
         <v>7</v>
       </c>
       <c r="C10" s="4">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>528</v>
       </c>
       <c r="D10" s="4">
@@ -1369,7 +1397,7 @@
         <v>10</v>
       </c>
       <c r="G10" s="4">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>30</v>
       </c>
     </row>
@@ -1378,7 +1406,8 @@
         <v>8</v>
       </c>
       <c r="C11" s="4">
-        <v>-900</v>
+        <f t="shared" si="2"/>
+        <v>627</v>
       </c>
       <c r="D11" s="4">
         <v>0.3</v>
@@ -1390,7 +1419,7 @@
         <v>11</v>
       </c>
       <c r="G11" s="4">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>33</v>
       </c>
     </row>
@@ -1399,7 +1428,7 @@
         <v>9</v>
       </c>
       <c r="C12" s="4">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>726</v>
       </c>
       <c r="D12" s="4">
@@ -1412,7 +1441,7 @@
         <v>12</v>
       </c>
       <c r="G12" s="4">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>36</v>
       </c>
     </row>
@@ -1421,7 +1450,7 @@
         <v>10</v>
       </c>
       <c r="C13" s="4">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>875</v>
       </c>
       <c r="D13" s="4">
@@ -1434,7 +1463,7 @@
         <v>13</v>
       </c>
       <c r="G13" s="4">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>39</v>
       </c>
     </row>
@@ -1443,7 +1472,7 @@
         <v>11</v>
       </c>
       <c r="C14" s="4">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>980</v>
       </c>
       <c r="D14" s="4">
@@ -1456,7 +1485,7 @@
         <v>14</v>
       </c>
       <c r="G14" s="4">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>42</v>
       </c>
     </row>
@@ -1465,7 +1494,7 @@
         <v>12</v>
       </c>
       <c r="C15" s="4">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>1085</v>
       </c>
       <c r="D15" s="4">
@@ -1478,7 +1507,7 @@
         <v>15</v>
       </c>
       <c r="G15" s="4">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>45</v>
       </c>
     </row>
@@ -1487,7 +1516,7 @@
         <v>13</v>
       </c>
       <c r="C16" s="4">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>1190</v>
       </c>
       <c r="D16" s="4">
@@ -1500,7 +1529,7 @@
         <v>16</v>
       </c>
       <c r="G16" s="4">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>48</v>
       </c>
     </row>
@@ -1509,7 +1538,7 @@
         <v>14</v>
       </c>
       <c r="C17" s="4">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>1295</v>
       </c>
       <c r="D17" s="4">
@@ -1522,7 +1551,7 @@
         <v>17</v>
       </c>
       <c r="G17" s="4">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>51</v>
       </c>
     </row>
@@ -1531,21 +1560,21 @@
         <v>15</v>
       </c>
       <c r="C18" s="4">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>1600</v>
       </c>
       <c r="D18" s="4">
         <v>1</v>
       </c>
       <c r="E18" s="4">
-        <f t="shared" ref="E18:E32" si="2">E17+30</f>
+        <f t="shared" ref="E18:E32" si="3">E17+30</f>
         <v>400</v>
       </c>
       <c r="F18" s="4">
         <v>18</v>
       </c>
       <c r="G18" s="4">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>54</v>
       </c>
     </row>
@@ -1554,21 +1583,21 @@
         <v>16</v>
       </c>
       <c r="C19" s="4">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>1720</v>
       </c>
       <c r="D19" s="4">
         <v>1</v>
       </c>
       <c r="E19" s="4">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>430</v>
       </c>
       <c r="F19" s="4">
         <v>19</v>
       </c>
       <c r="G19" s="4">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>57</v>
       </c>
     </row>
@@ -1577,21 +1606,21 @@
         <v>17</v>
       </c>
       <c r="C20" s="4">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>1840</v>
       </c>
       <c r="D20" s="4">
         <v>1</v>
       </c>
       <c r="E20" s="4">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>460</v>
       </c>
       <c r="F20" s="4">
         <v>20</v>
       </c>
       <c r="G20" s="4">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>60</v>
       </c>
     </row>
@@ -1600,21 +1629,21 @@
         <v>18</v>
       </c>
       <c r="C21" s="4">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>1960</v>
       </c>
       <c r="D21" s="4">
         <v>1</v>
       </c>
       <c r="E21" s="4">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>490</v>
       </c>
       <c r="F21" s="4">
         <v>21</v>
       </c>
       <c r="G21" s="4">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>63</v>
       </c>
     </row>
@@ -1623,21 +1652,21 @@
         <v>19</v>
       </c>
       <c r="C22" s="4">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>2080</v>
       </c>
       <c r="D22" s="4">
         <v>1</v>
       </c>
       <c r="E22" s="4">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>520</v>
       </c>
       <c r="F22" s="4">
         <v>22</v>
       </c>
       <c r="G22" s="4">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>66</v>
       </c>
     </row>
@@ -1646,21 +1675,21 @@
         <v>20</v>
       </c>
       <c r="C23" s="4">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>2200</v>
       </c>
       <c r="D23" s="4">
         <v>1</v>
       </c>
       <c r="E23" s="4">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>550</v>
       </c>
       <c r="F23" s="4">
         <v>23</v>
       </c>
       <c r="G23" s="4">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>69</v>
       </c>
     </row>
@@ -1669,21 +1698,21 @@
         <v>21</v>
       </c>
       <c r="C24" s="4">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>2610</v>
       </c>
       <c r="D24" s="4">
         <v>1.5</v>
       </c>
       <c r="E24" s="4">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>580</v>
       </c>
       <c r="F24" s="4">
         <v>24</v>
       </c>
       <c r="G24" s="4">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>72</v>
       </c>
     </row>
@@ -1692,21 +1721,21 @@
         <v>22</v>
       </c>
       <c r="C25" s="4">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>2745</v>
       </c>
       <c r="D25" s="4">
         <v>1.5</v>
       </c>
       <c r="E25" s="4">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>610</v>
       </c>
       <c r="F25" s="4">
         <v>25</v>
       </c>
       <c r="G25" s="4">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>75</v>
       </c>
     </row>
@@ -1715,21 +1744,21 @@
         <v>23</v>
       </c>
       <c r="C26" s="4">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>2880</v>
       </c>
       <c r="D26" s="4">
         <v>1.5</v>
       </c>
       <c r="E26" s="4">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>640</v>
       </c>
       <c r="F26" s="4">
         <v>26</v>
       </c>
       <c r="G26" s="4">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>78</v>
       </c>
     </row>
@@ -1738,21 +1767,21 @@
         <v>24</v>
       </c>
       <c r="C27" s="4">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>3015</v>
       </c>
       <c r="D27" s="4">
         <v>1.5</v>
       </c>
       <c r="E27" s="4">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>670</v>
       </c>
       <c r="F27" s="4">
         <v>27</v>
       </c>
       <c r="G27" s="4">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>81</v>
       </c>
     </row>
@@ -1761,21 +1790,21 @@
         <v>25</v>
       </c>
       <c r="C28" s="4">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>3150</v>
       </c>
       <c r="D28" s="4">
         <v>1.5</v>
       </c>
       <c r="E28" s="4">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>700</v>
       </c>
       <c r="F28" s="4">
         <v>28</v>
       </c>
       <c r="G28" s="4">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>84</v>
       </c>
     </row>
@@ -1784,21 +1813,21 @@
         <v>26</v>
       </c>
       <c r="C29" s="4">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>3285</v>
       </c>
       <c r="D29" s="4">
         <v>1.5</v>
       </c>
       <c r="E29" s="4">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>730</v>
       </c>
       <c r="F29" s="4">
         <v>29</v>
       </c>
       <c r="G29" s="4">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>87</v>
       </c>
     </row>
@@ -1807,21 +1836,21 @@
         <v>27</v>
       </c>
       <c r="C30" s="4">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>3420</v>
       </c>
       <c r="D30" s="4">
         <v>1.5</v>
       </c>
       <c r="E30" s="4">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>760</v>
       </c>
       <c r="F30" s="4">
         <v>30</v>
       </c>
       <c r="G30" s="4">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>90</v>
       </c>
     </row>
@@ -1830,21 +1859,21 @@
         <v>28</v>
       </c>
       <c r="C31" s="4">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>3950</v>
       </c>
       <c r="D31" s="4">
         <v>2</v>
       </c>
       <c r="E31" s="4">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>790</v>
       </c>
       <c r="F31" s="4">
         <v>31</v>
       </c>
       <c r="G31" s="4">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>93</v>
       </c>
     </row>
@@ -1853,21 +1882,21 @@
         <v>29</v>
       </c>
       <c r="C32" s="4">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>4100</v>
       </c>
       <c r="D32" s="4">
         <v>2</v>
       </c>
       <c r="E32" s="4">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>820</v>
       </c>
       <c r="F32" s="4">
         <v>32</v>
       </c>
       <c r="G32" s="4">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>96</v>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: implement Excel schema registry and serialization system using MemoryPack
</commit_message>
<xml_diff>
--- a/Documents/Excel/CityTest.xlsx
+++ b/Documents/Excel/CityTest.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\SeanProjects\CustomPackages\ExcelExtruder\Documents\Excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7967CBDD-0DA1-4A48-9CE0-026522295B83}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8D66C96E-CA4F-4D48-BEEA-4B04FA7B9873}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="783" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="783" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="sCityVO" sheetId="6" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="133" uniqueCount="108">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="127" uniqueCount="108">
   <si>
     <t>#</t>
   </si>
@@ -369,7 +369,7 @@
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
-    <t>Map12</t>
+    <t>Map2</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
 </sst>
@@ -738,7 +738,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6B4CF102-FCD0-4C03-97A2-6BA18FF3CB38}">
-  <dimension ref="A1:G20"/>
+  <dimension ref="A1:G19"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="3.25" style="3" customWidth="1"/>
@@ -1140,26 +1140,6 @@
       </c>
       <c r="G19" s="4" t="s">
         <v>104</v>
-      </c>
-    </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="B20" s="4" t="s">
-        <v>106</v>
-      </c>
-      <c r="C20" s="4" t="s">
-        <v>40</v>
-      </c>
-      <c r="D20" s="4" t="s">
-        <v>41</v>
-      </c>
-      <c r="E20" s="4" t="s">
-        <v>42</v>
-      </c>
-      <c r="F20" s="4" t="s">
-        <v>81</v>
-      </c>
-      <c r="G20" s="4" t="s">
-        <v>90</v>
       </c>
     </row>
   </sheetData>

</xml_diff>